<commit_message>
atualizando casos de teste
</commit_message>
<xml_diff>
--- a/documentação/Testes/Caso de Teste/UC05 - HISTÓRICO DE CONSULTA DE PACIENTE.xlsx
+++ b/documentação/Testes/Caso de Teste/UC05 - HISTÓRICO DE CONSULTA DE PACIENTE.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
   <si>
     <t xml:space="preserve">Caso de Teste</t>
   </si>
@@ -56,6 +56,9 @@
     <t xml:space="preserve">Sistema exibe lista de consultas com campos: Paciente, Horário, Dia, Especialista, Especialidade, Clínica, Status, Botão "Avaliar" (se status="Realizada").</t>
   </si>
   <si>
+    <t xml:space="preserve">OK</t>
+  </si>
+  <si>
     <t xml:space="preserve">melhoria, na tela trocar medico por Especialista</t>
   </si>
   <si>
@@ -69,9 +72,6 @@
   </si>
   <si>
     <t xml:space="preserve">“Não há consultas realizadas.”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK</t>
   </si>
   <si>
     <t xml:space="preserve">CT03 - Avaliação de Consulta (Sucesso)</t>
@@ -298,13 +298,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H1048576"/>
-  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.01"/>
@@ -339,7 +445,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
@@ -352,33 +458,36 @@
       <c r="D2" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="G2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -392,7 +501,7 @@
         <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H4" s="6"/>
     </row>
@@ -431,7 +540,7 @@
         <v>30</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H6" s="6"/>
     </row>
@@ -449,7 +558,7 @@
         <v>34</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H7" s="6"/>
     </row>
@@ -467,7 +576,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H8" s="6"/>
     </row>
@@ -485,7 +594,7 @@
         <v>42</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H9" s="6"/>
     </row>

</xml_diff>